<commit_message>
Update town data 2026-09-13T23:21:10Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-12T23:10:13Z</t>
+          <t>2026-09-13T23:21:10Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-12T23:10:13Z</t>
+          <t>2026-09-13T23:21:10Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-12T23:10:13Z</t>
+          <t>2026-09-13T23:21:10Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-14T23:56:49Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-13T23:21:10Z</t>
+          <t>2026-09-14T23:56:49Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-13T23:21:10Z</t>
+          <t>2026-09-14T23:56:49Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-13T23:21:10Z</t>
+          <t>2026-09-14T23:56:49Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-15T23:35:34Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-14T23:56:49Z</t>
+          <t>2026-09-15T23:35:34Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-14T23:56:49Z</t>
+          <t>2026-09-15T23:35:34Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-14T23:56:49Z</t>
+          <t>2026-09-15T23:35:34Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-16T23:44:15Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-15T23:35:34Z</t>
+          <t>2026-09-16T23:44:15Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-15T23:35:34Z</t>
+          <t>2026-09-16T23:44:15Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-15T23:35:34Z</t>
+          <t>2026-09-16T23:44:15Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-17T23:36:55Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-16T23:44:15Z</t>
+          <t>2026-09-17T23:36:55Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-16T23:44:15Z</t>
+          <t>2026-09-17T23:36:55Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-16T23:44:15Z</t>
+          <t>2026-09-17T23:36:55Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-18T23:29:24Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-17T23:36:55Z</t>
+          <t>2026-09-18T23:29:24Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-17T23:36:55Z</t>
+          <t>2026-09-18T23:29:24Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-17T23:36:55Z</t>
+          <t>2026-09-18T23:29:24Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-19T23:21:32Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-18T23:29:24Z</t>
+          <t>2026-09-19T23:21:32Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-18T23:29:24Z</t>
+          <t>2026-09-19T23:21:32Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-18T23:29:24Z</t>
+          <t>2026-09-19T23:21:32Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-20T23:22:02Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-19T23:21:32Z</t>
+          <t>2026-09-20T23:22:02Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-19T23:21:32Z</t>
+          <t>2026-09-20T23:22:02Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-19T23:21:32Z</t>
+          <t>2026-09-20T23:22:02Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-22T00:14:16Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-20T23:22:02Z</t>
+          <t>2026-09-22T00:14:16Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-20T23:22:02Z</t>
+          <t>2026-09-22T00:14:16Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-20T23:22:02Z</t>
+          <t>2026-09-22T00:14:16Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-22T23:43:11Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-22T00:14:16Z</t>
+          <t>2026-09-22T23:43:11Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-22T00:14:16Z</t>
+          <t>2026-09-22T23:43:11Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-22T00:14:16Z</t>
+          <t>2026-09-22T23:43:11Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-23T23:52:33Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-22T23:43:11Z</t>
+          <t>2026-09-23T23:52:33Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-22T23:43:11Z</t>
+          <t>2026-09-23T23:52:33Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-22T23:43:11Z</t>
+          <t>2026-09-23T23:52:33Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-24T23:57:38Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-23T23:52:33Z</t>
+          <t>2026-09-24T23:57:38Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-23T23:52:33Z</t>
+          <t>2026-09-24T23:57:38Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-23T23:52:33Z</t>
+          <t>2026-09-24T23:57:38Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-26T00:00:53Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-24T23:57:38Z</t>
+          <t>2026-09-26T00:00:53Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-24T23:57:38Z</t>
+          <t>2026-09-26T00:00:53Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-24T23:57:38Z</t>
+          <t>2026-09-26T00:00:53Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-26T23:45:30Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-26T00:00:53Z</t>
+          <t>2026-09-26T23:45:30Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-26T00:00:53Z</t>
+          <t>2026-09-26T23:45:30Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-26T00:00:53Z</t>
+          <t>2026-09-26T23:45:30Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-27T23:52:34Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-26T23:45:30Z</t>
+          <t>2026-09-27T23:52:34Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-26T23:45:30Z</t>
+          <t>2026-09-27T23:52:34Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-26T23:45:30Z</t>
+          <t>2026-09-27T23:52:34Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-29T01:09:30Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-27T23:52:34Z</t>
+          <t>2026-09-29T01:09:30Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-27T23:52:34Z</t>
+          <t>2026-09-29T01:09:30Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-27T23:52:34Z</t>
+          <t>2026-09-29T01:09:30Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-09-30T00:40:29Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-29T01:09:30Z</t>
+          <t>2026-09-30T00:40:28Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-29T01:09:30Z</t>
+          <t>2026-09-30T00:40:28Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-29T01:09:30Z</t>
+          <t>2026-09-30T00:40:28Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-01T00:42:29Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-30T00:40:28Z</t>
+          <t>2026-10-01T00:42:29Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-30T00:40:28Z</t>
+          <t>2026-10-01T00:42:29Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-30T00:40:28Z</t>
+          <t>2026-10-01T00:42:29Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-02T01:01:56Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-01T00:42:29Z</t>
+          <t>2026-10-02T01:01:56Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-01T00:42:29Z</t>
+          <t>2026-10-02T01:01:56Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-01T00:42:29Z</t>
+          <t>2026-10-02T01:01:56Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-03T00:37:50Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -437,7 +437,7 @@
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
@@ -537,12 +537,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3f8b50970523ea07f1a945df0c376d049901799e</t>
+          <t>88217d6344811610e83f618cc8318c3b39052e41</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Madhu Hospital</t>
+          <t>KRISHNA HOSPITAL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -553,26 +553,22 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>D.No.21/110, SKD colony, Road No-1, Adoni, Kurnool</t>
+          <t>21/63, S.K.D COLONY  , ADONI KURNOOL ANDHRA PRADESH</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>D.No.21/110, SKD colony, Road No-1, Adoni, Kurnool</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>518301</t>
-        </is>
-      </c>
+          <t>21/63, S.K.D COLONY  , ADONI KURNOOL ANDHRA PRADESH</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>ADONI</t>
+          <t>Adoni</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -584,12 +580,12 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>insurer_star_health</t>
+          <t>insurer_hdfc_ergo</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-02T01:01:56Z</t>
+          <t>2026-10-03T00:37:50Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -597,12 +593,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>88217d6344811610e83f618cc8318c3b39052e41</t>
+          <t>1b20c61cd98fd7e85ff2438679ac54e899d06fb7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>KRISHNA HOSPITAL</t>
+          <t>RAGHVENDRA EYE CARE HOSPITAL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -613,12 +609,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>21/63, S.K.D COLONY  , ADONI KURNOOL ANDHRA PRADESH</t>
+          <t>21/63-1 1ST FLOOR ABOVE KRISHNA HOSPITAL  , ABOVE KRISHNA HOSPITAL KURNOOL ANDHRA PRADESH</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>21/63, S.K.D COLONY  , ADONI KURNOOL ANDHRA PRADESH</t>
+          <t>21/63-1 1ST FLOOR ABOVE KRISHNA HOSPITAL  , ABOVE KRISHNA HOSPITAL KURNOOL ANDHRA PRADESH</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -645,66 +641,10 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-02T01:01:56Z</t>
+          <t>2026-10-03T00:37:50Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1b20c61cd98fd7e85ff2438679ac54e899d06fb7</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>RAGHVENDRA EYE CARE HOSPITAL</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Hospital</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>21/63-1 1ST FLOOR ABOVE KRISHNA HOSPITAL  , ABOVE KRISHNA HOSPITAL KURNOOL ANDHRA PRADESH</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>21/63-1 1ST FLOOR ABOVE KRISHNA HOSPITAL  , ABOVE KRISHNA HOSPITAL KURNOOL ANDHRA PRADESH</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Adoni</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Andhra Pradesh</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>insurer_hdfc_ergo</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-10-02T01:01:56Z</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update town data 2026-10-03T23:58:48Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -437,7 +437,7 @@
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
@@ -537,12 +537,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>88217d6344811610e83f618cc8318c3b39052e41</t>
+          <t>3f8b50970523ea07f1a945df0c376d049901799e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KRISHNA HOSPITAL</t>
+          <t>Madhu Hospital</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -553,22 +553,26 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>21/63, S.K.D COLONY  , ADONI KURNOOL ANDHRA PRADESH</t>
+          <t>D.No.21/110, SKD colony, Road No-1, Adoni, Kurnool</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>21/63, S.K.D COLONY  , ADONI KURNOOL ANDHRA PRADESH</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>D.No.21/110, SKD colony, Road No-1, Adoni, Kurnool</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>518301</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Adoni</t>
+          <t>ADONI</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -580,12 +584,12 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>insurer_hdfc_ergo</t>
+          <t>insurer_star_health</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-03T00:37:50Z</t>
+          <t>2026-10-03T23:58:48Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -593,12 +597,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1b20c61cd98fd7e85ff2438679ac54e899d06fb7</t>
+          <t>88217d6344811610e83f618cc8318c3b39052e41</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RAGHVENDRA EYE CARE HOSPITAL</t>
+          <t>KRISHNA HOSPITAL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -609,12 +613,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>21/63-1 1ST FLOOR ABOVE KRISHNA HOSPITAL  , ABOVE KRISHNA HOSPITAL KURNOOL ANDHRA PRADESH</t>
+          <t>21/63, S.K.D COLONY  , ADONI KURNOOL ANDHRA PRADESH</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>21/63-1 1ST FLOOR ABOVE KRISHNA HOSPITAL  , ABOVE KRISHNA HOSPITAL KURNOOL ANDHRA PRADESH</t>
+          <t>21/63, S.K.D COLONY  , ADONI KURNOOL ANDHRA PRADESH</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -641,10 +645,66 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-03T00:37:50Z</t>
+          <t>2026-10-03T23:58:48Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1b20c61cd98fd7e85ff2438679ac54e899d06fb7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RAGHVENDRA EYE CARE HOSPITAL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>21/63-1 1ST FLOOR ABOVE KRISHNA HOSPITAL  , ABOVE KRISHNA HOSPITAL KURNOOL ANDHRA PRADESH</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>21/63-1 1ST FLOOR ABOVE KRISHNA HOSPITAL  , ABOVE KRISHNA HOSPITAL KURNOOL ANDHRA PRADESH</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Adoni</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>insurer_hdfc_ergo</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-10-03T23:58:48Z</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update town data 2026-10-05T00:04:41Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-03T23:58:48Z</t>
+          <t>2026-10-05T00:04:40Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-03T23:58:48Z</t>
+          <t>2026-10-05T00:04:40Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-03T23:58:48Z</t>
+          <t>2026-10-05T00:04:40Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-06T01:49:56Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-05T00:04:40Z</t>
+          <t>2026-10-06T01:49:56Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-05T00:04:40Z</t>
+          <t>2026-10-06T01:49:56Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-05T00:04:40Z</t>
+          <t>2026-10-06T01:49:56Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-07T00:55:04Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-06T01:49:56Z</t>
+          <t>2026-10-07T00:55:03Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-06T01:49:56Z</t>
+          <t>2026-10-07T00:55:03Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-06T01:49:56Z</t>
+          <t>2026-10-07T00:55:03Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-08T01:11:47Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-07T00:55:03Z</t>
+          <t>2026-10-08T01:11:47Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-07T00:55:03Z</t>
+          <t>2026-10-08T01:11:47Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-07T00:55:03Z</t>
+          <t>2026-10-08T01:11:47Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-09T01:19:51Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-08T01:11:47Z</t>
+          <t>2026-10-09T01:19:51Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-08T01:11:47Z</t>
+          <t>2026-10-09T01:19:51Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-08T01:11:47Z</t>
+          <t>2026-10-09T01:19:51Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-10T01:07:38Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-09T01:19:51Z</t>
+          <t>2026-10-10T01:07:38Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-09T01:19:51Z</t>
+          <t>2026-10-10T01:07:38Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-09T01:19:51Z</t>
+          <t>2026-10-10T01:07:38Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-11T00:20:49Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-10T01:07:38Z</t>
+          <t>2026-10-11T00:20:49Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-10T01:07:38Z</t>
+          <t>2026-10-11T00:20:49Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-10T01:07:38Z</t>
+          <t>2026-10-11T00:20:49Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-12T00:41:21Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-11T00:20:49Z</t>
+          <t>2026-10-12T00:41:21Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-11T00:20:49Z</t>
+          <t>2026-10-12T00:41:21Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-11T00:20:49Z</t>
+          <t>2026-10-12T00:41:21Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-13T02:40:40Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -429,7 +429,7 @@
     <col width="57" customWidth="1" min="5" max="5"/>
     <col width="57" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
@@ -437,7 +437,7 @@
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-12T00:41:21Z</t>
+          <t>2026-10-13T02:40:39Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-12T00:41:21Z</t>
+          <t>2026-10-13T02:40:39Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,10 +701,74 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-12T00:41:21Z</t>
+          <t>2026-10-13T02:40:39Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8fbc6cd8f74a0d537335decbfc01d50f3c120eda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Madhu Hospital</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>21-111/112, Skd Colony Road No-1, Behind Nirmal Talkies</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>21-111/112, Skd Colony Road No-1, Behind Nirmal Talkies</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>518301</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>09491897369</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Adoni</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>insurer_icici_lombard</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-10-13T02:40:39Z</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update town data 2026-10-14T00:29:37Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-13T02:40:39Z</t>
+          <t>2026-10-14T00:29:37Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-13T02:40:39Z</t>
+          <t>2026-10-14T00:29:37Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-13T02:40:39Z</t>
+          <t>2026-10-14T00:29:37Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-13T02:40:39Z</t>
+          <t>2026-10-14T00:29:37Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-15T00:01:50Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-14T00:29:37Z</t>
+          <t>2026-10-15T00:01:50Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-14T00:29:37Z</t>
+          <t>2026-10-15T00:01:50Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-14T00:29:37Z</t>
+          <t>2026-10-15T00:01:50Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-14T00:29:37Z</t>
+          <t>2026-10-15T00:01:50Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-15T23:46:00Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-15T00:01:50Z</t>
+          <t>2026-10-15T23:46:00Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-15T00:01:50Z</t>
+          <t>2026-10-15T23:46:00Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-15T00:01:50Z</t>
+          <t>2026-10-15T23:46:00Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-15T00:01:50Z</t>
+          <t>2026-10-15T23:46:00Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-16T23:46:15Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-15T23:46:00Z</t>
+          <t>2026-10-16T23:46:15Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-15T23:46:00Z</t>
+          <t>2026-10-16T23:46:15Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-15T23:46:00Z</t>
+          <t>2026-10-16T23:46:15Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-15T23:46:00Z</t>
+          <t>2026-10-16T23:46:15Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-17T23:19:00Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -429,7 +429,7 @@
     <col width="57" customWidth="1" min="5" max="5"/>
     <col width="57" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
@@ -437,7 +437,7 @@
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-16T23:46:15Z</t>
+          <t>2026-10-17T23:19:00Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-16T23:46:15Z</t>
+          <t>2026-10-17T23:19:00Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,74 +701,10 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-16T23:46:15Z</t>
+          <t>2026-10-17T23:19:00Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>8fbc6cd8f74a0d537335decbfc01d50f3c120eda</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Madhu Hospital</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Hospital</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>21-111/112, Skd Colony Road No-1, Behind Nirmal Talkies</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>21-111/112, Skd Colony Road No-1, Behind Nirmal Talkies</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>518301</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>09491897369</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Adoni</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Andhra Pradesh</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>insurer_icici_lombard</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-10-16T23:46:15Z</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update town data 2026-10-18T23:32:28Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -429,7 +429,7 @@
     <col width="57" customWidth="1" min="5" max="5"/>
     <col width="57" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
@@ -437,7 +437,7 @@
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-17T23:19:00Z</t>
+          <t>2026-10-18T23:32:28Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-17T23:19:00Z</t>
+          <t>2026-10-18T23:32:28Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,10 +701,74 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-17T23:19:00Z</t>
+          <t>2026-10-18T23:32:28Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8fbc6cd8f74a0d537335decbfc01d50f3c120eda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Madhu Hospital</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>21-111/112, Skd Colony Road No-1, Behind Nirmal Talkies</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>21-111/112, Skd Colony Road No-1, Behind Nirmal Talkies</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>518301</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>09491897369</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Adoni</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>insurer_icici_lombard</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-10-18T23:32:28Z</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update town data 2026-10-20T00:31:54Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-18T23:32:28Z</t>
+          <t>2026-10-20T00:31:54Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-18T23:32:28Z</t>
+          <t>2026-10-20T00:31:54Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-18T23:32:28Z</t>
+          <t>2026-10-20T00:31:54Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-18T23:32:28Z</t>
+          <t>2026-10-20T00:31:54Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-21T00:01:50Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-20T00:31:54Z</t>
+          <t>2026-10-21T00:01:50Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-20T00:31:54Z</t>
+          <t>2026-10-21T00:01:50Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-20T00:31:54Z</t>
+          <t>2026-10-21T00:01:50Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-20T00:31:54Z</t>
+          <t>2026-10-21T00:01:50Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-22T00:07:19Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-21T00:01:50Z</t>
+          <t>2026-10-22T00:07:19Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-21T00:01:50Z</t>
+          <t>2026-10-22T00:07:19Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-21T00:01:50Z</t>
+          <t>2026-10-22T00:07:19Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-21T00:01:50Z</t>
+          <t>2026-10-22T00:07:19Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-23T00:04:59Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-22T00:07:19Z</t>
+          <t>2026-10-23T00:04:59Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-22T00:07:19Z</t>
+          <t>2026-10-23T00:04:59Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-22T00:07:19Z</t>
+          <t>2026-10-23T00:04:59Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-22T00:07:19Z</t>
+          <t>2026-10-23T00:04:59Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-23T23:55:25Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-23T00:04:59Z</t>
+          <t>2026-10-23T23:55:25Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-23T00:04:59Z</t>
+          <t>2026-10-23T23:55:25Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-23T00:04:59Z</t>
+          <t>2026-10-23T23:55:25Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-23T00:04:59Z</t>
+          <t>2026-10-23T23:55:25Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-24T23:32:49Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:55:25Z</t>
+          <t>2026-10-24T23:32:49Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-23T23:55:25Z</t>
+          <t>2026-10-24T23:32:49Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:55:25Z</t>
+          <t>2026-10-24T23:32:49Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-23T23:55:25Z</t>
+          <t>2026-10-24T23:32:49Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-25T23:27:57Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-24T23:32:49Z</t>
+          <t>2026-10-25T23:27:57Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-24T23:32:49Z</t>
+          <t>2026-10-25T23:27:57Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-24T23:32:49Z</t>
+          <t>2026-10-25T23:27:57Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-24T23:32:49Z</t>
+          <t>2026-10-25T23:27:57Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-27T00:41:50Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-25T23:27:57Z</t>
+          <t>2026-10-27T00:41:50Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-25T23:27:57Z</t>
+          <t>2026-10-27T00:41:50Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-25T23:27:57Z</t>
+          <t>2026-10-27T00:41:50Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-25T23:27:57Z</t>
+          <t>2026-10-27T00:41:50Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-28T00:39:26Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-27T00:41:50Z</t>
+          <t>2026-10-28T00:39:26Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-27T00:41:50Z</t>
+          <t>2026-10-28T00:39:26Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-27T00:41:50Z</t>
+          <t>2026-10-28T00:39:26Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-27T00:41:50Z</t>
+          <t>2026-10-28T00:39:26Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-29T01:09:04Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-28T00:39:26Z</t>
+          <t>2026-10-29T01:09:04Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-28T00:39:26Z</t>
+          <t>2026-10-29T01:09:04Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-28T00:39:26Z</t>
+          <t>2026-10-29T01:09:04Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-28T00:39:26Z</t>
+          <t>2026-10-29T01:09:04Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-30T01:16:07Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-29T01:09:04Z</t>
+          <t>2026-10-30T01:16:07Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-29T01:09:04Z</t>
+          <t>2026-10-30T01:16:07Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-29T01:09:04Z</t>
+          <t>2026-10-30T01:16:07Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-29T01:09:04Z</t>
+          <t>2026-10-30T01:16:07Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update town data 2026-10-31T00:57:36Z
</commit_message>
<xml_diff>
--- a/data/adoni_directory.xlsx
+++ b/data/adoni_directory.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:16:07Z</t>
+          <t>2026-10-31T00:57:36Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-10-30T01:16:07Z</t>
+          <t>2026-10-31T00:57:36Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:16:07Z</t>
+          <t>2026-10-31T00:57:36Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-10-30T01:16:07Z</t>
+          <t>2026-10-31T00:57:36Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>

</xml_diff>